<commit_message>
2.4 Dxf for autocrease
</commit_message>
<xml_diff>
--- a/Fusion360/RightingArmSweep_cleaned_plotted.xlsx
+++ b/Fusion360/RightingArmSweep_cleaned_plotted.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jakob\Documents\GitHub\Folding-kayak\Fusion360\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8158D7F8-A872-4DCF-AA6D-7B826D8ED8F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05AE5B08-684A-4287-9294-E7497B43FAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{DE637436-0473-404C-BC50-937410BA525C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{DE637436-0473-404C-BC50-937410BA525C}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData_v3_comp" sheetId="2" r:id="rId1"/>
     <sheet name="TestData_v3_comp (2)" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">TestData_v3_comp!$A$1:$G$17</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">TestData_v3_comp!$A$1:$G$15</definedName>
     <definedName name="ExternalData_1" localSheetId="1" hidden="1">'TestData_v3_comp (2)'!$A$1:$H$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="9">
   <si>
     <t>HeelAngle</t>
   </si>
@@ -80,6 +80,9 @@
   <si>
     <t>Nm 90kg v3</t>
   </si>
+  <si>
+    <t>v2.4_68</t>
+  </si>
 </sst>
 </file>
 
@@ -94,15 +97,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor theme="9" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -110,17 +119,97 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="9" tint="0.79998168889431442"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -197,10 +286,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$A$2:$A$17</c:f>
+              <c:f>TestData_v3_comp!$A$2:$A$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -226,27 +315,21 @@
                   <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>15</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>16</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>18</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>20</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>22</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>26</c:v>
                 </c:pt>
               </c:numCache>
@@ -254,10 +337,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$B$2:$B$17</c:f>
+              <c:f>TestData_v3_comp!$B$2:$B$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -282,22 +365,22 @@
                 <c:pt idx="7">
                   <c:v>26.386600348392697</c:v>
                 </c:pt>
+                <c:pt idx="8">
+                  <c:v>29.492855410981377</c:v>
+                </c:pt>
                 <c:pt idx="9">
-                  <c:v>29.492855410981377</c:v>
+                  <c:v>31.876605800476643</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>31.876605800476643</c:v>
+                  <c:v>33.665694816156972</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>33.665694816156972</c:v>
+                  <c:v>34.955435729999998</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>34.955435729999998</c:v>
+                  <c:v>35.820851562722908</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>35.820851562722908</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>36.078511490621082</c:v>
                 </c:pt>
               </c:numCache>
@@ -350,80 +433,47 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$A$2:$A$17</c:f>
+              <c:f>TestData_v3_comp!$A$20:$A$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>18</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>22</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="14">
                   <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>26</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$C$2:$C$17</c:f>
+              <c:f>TestData_v3_comp!$C$20:$C$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="1">
                   <c:v>14.325600000000001</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="2">
                   <c:v>20.116800000000001</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="3">
                   <c:v>20.421600000000002</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="4">
                   <c:v>17.3736</c:v>
                 </c:pt>
               </c:numCache>
@@ -476,10 +526,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$A$2:$A$17</c:f>
+              <c:f>TestData_v3_comp!$A$2:$A$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -505,27 +555,21 @@
                   <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>15</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>16</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>18</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>20</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>22</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>26</c:v>
                 </c:pt>
               </c:numCache>
@@ -533,10 +577,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$D$2:$D$17</c:f>
+              <c:f>TestData_v3_comp!$D$2:$D$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -561,22 +605,22 @@
                 <c:pt idx="7">
                   <c:v>3.4316156461438929</c:v>
                 </c:pt>
+                <c:pt idx="8">
+                  <c:v>3.6244941391413121</c:v>
+                </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.6244941391413121</c:v>
+                  <c:v>3.5814365777583035</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3.5814365777583035</c:v>
+                  <c:v>3.345700169036423</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.345700169036423</c:v>
+                  <c:v>2.9564879576701841</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.9564879576701841</c:v>
+                  <c:v>2.4498664614607613</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.4498664614607613</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>1.8595618939661129</c:v>
                 </c:pt>
               </c:numCache>
@@ -629,10 +673,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$A$2:$A$17</c:f>
+              <c:f>TestData_v3_comp!$A$2:$A$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -658,27 +702,21 @@
                   <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>15</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>16</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>18</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>20</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>22</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>26</c:v>
                 </c:pt>
               </c:numCache>
@@ -686,10 +724,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$E$2:$E$17</c:f>
+              <c:f>TestData_v3_comp!$E$2:$E$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -714,22 +752,22 @@
                 <c:pt idx="7">
                   <c:v>8.6821226642829519</c:v>
                 </c:pt>
+                <c:pt idx="8">
+                  <c:v>8.5778441065895183</c:v>
+                </c:pt>
                 <c:pt idx="9">
-                  <c:v>8.5778441065895183</c:v>
+                  <c:v>8.2172795945172261</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>8.2172795945172261</c:v>
+                  <c:v>7.6472604719564963</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>7.6472604719564963</c:v>
+                  <c:v>6.9099309450000002</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>6.9099309450000002</c:v>
+                  <c:v>6.0438475571111816</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>6.0438475571111816</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>5.0848986300286292</c:v>
                 </c:pt>
               </c:numCache>
@@ -782,10 +820,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$A$2:$A$17</c:f>
+              <c:f>TestData_v3_comp!$A$2:$A$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -811,27 +849,21 @@
                   <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>15</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>16</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>18</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>20</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>22</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>26</c:v>
                 </c:pt>
               </c:numCache>
@@ -839,10 +871,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$F$2:$F$17</c:f>
+              <c:f>TestData_v3_comp!$F$2:$F$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -867,22 +899,22 @@
                 <c:pt idx="7">
                   <c:v>36.968044839999997</c:v>
                 </c:pt>
+                <c:pt idx="8">
+                  <c:v>39.486924298506949</c:v>
+                </c:pt>
                 <c:pt idx="9">
-                  <c:v>39.486924298506949</c:v>
+                  <c:v>41.299882744762179</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>41.299882744762179</c:v>
+                  <c:v>42.527524768893407</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>42.527524768893407</c:v>
+                  <c:v>43.271801437912231</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>43.271801437912231</c:v>
+                  <c:v>43.615839341589606</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>43.615839341589606</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>43.628240126287153</c:v>
                 </c:pt>
               </c:numCache>
@@ -935,80 +967,47 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$A$2:$A$17</c:f>
+              <c:f>TestData_v3_comp!$A$20:$A$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>18</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>22</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="14">
                   <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>26</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>TestData_v3_comp!$G$2:$G$17</c:f>
+              <c:f>TestData_v3_comp!$G$20:$G$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="1">
                   <c:v>24.688800000000001</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="2">
                   <c:v>30.1752</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="3">
                   <c:v>31.089600000000001</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="4">
                   <c:v>28.956</c:v>
                 </c:pt>
               </c:numCache>
@@ -1018,6 +1017,105 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000005-B58B-4634-8CC9-5AEE2848D89C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>TestData_v3_comp!$H$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>v2.4_68</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>TestData_v3_comp!$A$20:$A$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>25</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>TestData_v3_comp!$H$20:$H$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>16.47</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>16.975000000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>16.344000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9F54-4169-BA88-D9ED5881FF25}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1317,7 +1415,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="nb-NO"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2887,16 +2985,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>666750</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>870857</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>138112</xdr:rowOff>
+      <xdr:rowOff>54429</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>23812</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>81642</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>122465</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2969,8 +3067,8 @@
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" connectionId="1" xr16:uid="{FC54B80C-80D3-4D71-B7A1-FC6EFCF51274}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
-  <queryTableRefresh nextId="9">
-    <queryTableFields count="7">
+  <queryTableRefresh nextId="10" unboundColumnsRight="1">
+    <queryTableFields count="8">
       <queryTableField id="1" name="HeelAngle" tableColumnId="1"/>
       <queryTableField id="2" name="30.09.2026_v3_90.72kg_10in+30mm_fromK" tableColumnId="2"/>
       <queryTableField id="3" name="Solo microbootlegger w 90.72kg 10 in ab seat" tableColumnId="3"/>
@@ -2978,6 +3076,7 @@
       <queryTableField id="5" name="V2_asbuilt_68.04kg_10in30mmK" tableColumnId="5"/>
       <queryTableField id="6" name="V3_68.04kg_10in30mmK" tableColumnId="6"/>
       <queryTableField id="7" name="Solo Microboot" tableColumnId="7"/>
+      <queryTableField id="9" dataBound="0" tableColumnId="8"/>
     </queryTableFields>
     <queryTableDeletedFields count="1">
       <deletedField name="Column1"/>
@@ -3007,16 +3106,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2CB759EE-43C6-43CC-9D2F-52FDF7324CF4}" name="TestData_v3_comp" displayName="TestData_v3_comp" ref="A1:G18" tableType="queryTable" totalsRowCount="1">
-  <autoFilter ref="A1:G17" xr:uid="{2CB759EE-43C6-43CC-9D2F-52FDF7324CF4}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{8EE95E13-EDCD-45A0-92A5-D366ADF85B4F}" uniqueName="1" name="HeelAngle" queryTableFieldId="1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2CB759EE-43C6-43CC-9D2F-52FDF7324CF4}" name="TestData_v3_comp" displayName="TestData_v3_comp" ref="A1:H16" tableType="queryTable" totalsRowCount="1">
+  <autoFilter ref="A1:H15" xr:uid="{2CB759EE-43C6-43CC-9D2F-52FDF7324CF4}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{8EE95E13-EDCD-45A0-92A5-D366ADF85B4F}" uniqueName="1" name="HeelAngle" queryTableFieldId="1" totalsRowDxfId="0"/>
     <tableColumn id="2" xr3:uid="{126E497A-636B-4139-88F3-596BA239455E}" uniqueName="2" name="30.09.2026_v3_90.72kg_10in+30mm_fromK" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{09E9EAF0-44C4-4FE3-A4D9-9473C26B8064}" uniqueName="3" name="Solo Microboot 200p" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{81A208C9-F420-4AB9-AC07-EC220E07CBC1}" uniqueName="4" name="V2_asbuilt_90.72kg_10in30mm" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{FB6AE0FC-3347-4D9D-AECB-95935DCFF936}" uniqueName="5" name="V2_asbuilt_68.04kg_10in30mmK" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{5F942661-89C4-41BE-AFE0-16EA42FD3741}" uniqueName="6" name="V3_68.04kg_10in30mmK" queryTableFieldId="6"/>
     <tableColumn id="7" xr3:uid="{6EC271AA-EBEA-4661-968E-967AC1E0B5CB}" uniqueName="7" name="Solo Microboot 150p2" queryTableFieldId="7"/>
+    <tableColumn id="8" xr3:uid="{D842E034-B767-4CEB-9FA3-A71B5519825B}" uniqueName="8" name="v2.4_68" queryTableFieldId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3027,7 +3127,7 @@
   <autoFilter ref="A1:H15" xr:uid="{2CB759EE-43C6-43CC-9D2F-52FDF7324CF4}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{6E2A9D4C-F337-4EAC-B601-C7DFBB284A73}" uniqueName="1" name="HeelAngle" queryTableFieldId="1"/>
-    <tableColumn id="9" xr3:uid="{81DCFCC1-6CB6-4769-9550-A887B2718498}" uniqueName="9" name="Nm 90kg v3" queryTableFieldId="9" dataDxfId="0">
+    <tableColumn id="9" xr3:uid="{81DCFCC1-6CB6-4769-9550-A887B2718498}" uniqueName="9" name="Nm 90kg v3" queryTableFieldId="9" dataDxfId="1">
       <calculatedColumnFormula>C2*90.72*9.82/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{46AAE8FD-1101-47CB-AC78-7D86C3E61431}" uniqueName="2" name="30.09.2026_v3_90.72kg_10in+30mm_fromK" queryTableFieldId="2"/>
@@ -3360,7 +3460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68A1FCED-64A4-4DF4-8B61-BDD029044CE0}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
@@ -3372,7 +3472,7 @@
     <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3394,8 +3494,11 @@
       <c r="G1" t="s">
         <v>5</v>
       </c>
+      <c r="H1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -3418,7 +3521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3435,7 +3538,7 @@
         <v>5.7767789695848091</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4</v>
       </c>
@@ -3452,7 +3555,7 @@
         <v>11.579616759976219</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>6</v>
       </c>
@@ -3469,7 +3572,7 @@
         <v>17.43444212378887</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>8</v>
       </c>
@@ -3486,7 +3589,7 @@
         <v>23.367199814525371</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>10</v>
       </c>
@@ -3510,7 +3613,7 @@
         <v>24.688800000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>12</v>
       </c>
@@ -3527,7 +3630,7 @@
         <v>33.566160253357296</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>14</v>
       </c>
@@ -3544,134 +3647,205 @@
         <v>36.968044839999997</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
+        <v>16</v>
+      </c>
+      <c r="B10">
+        <v>29.492855410981377</v>
+      </c>
+      <c r="D10">
+        <v>3.6244941391413121</v>
+      </c>
+      <c r="E10">
+        <v>8.5778441065895183</v>
+      </c>
+      <c r="F10">
+        <v>39.486924298506949</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>18</v>
+      </c>
+      <c r="B11">
+        <v>31.876605800476643</v>
+      </c>
+      <c r="D11">
+        <v>3.5814365777583035</v>
+      </c>
+      <c r="E11">
+        <v>8.2172795945172261</v>
+      </c>
+      <c r="F11">
+        <v>41.299882744762179</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>20</v>
+      </c>
+      <c r="B12">
+        <v>33.665694816156972</v>
+      </c>
+      <c r="C12">
+        <v>20.421600000000002</v>
+      </c>
+      <c r="D12">
+        <v>3.345700169036423</v>
+      </c>
+      <c r="E12">
+        <v>7.6472604719564963</v>
+      </c>
+      <c r="F12">
+        <v>42.527524768893407</v>
+      </c>
+      <c r="G12">
+        <v>31.089600000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>22</v>
+      </c>
+      <c r="B13">
+        <v>34.955435729999998</v>
+      </c>
+      <c r="D13">
+        <v>2.9564879576701841</v>
+      </c>
+      <c r="E13">
+        <v>6.9099309450000002</v>
+      </c>
+      <c r="F13">
+        <v>43.271801437912231</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>24</v>
+      </c>
+      <c r="B14">
+        <v>35.820851562722908</v>
+      </c>
+      <c r="D14">
+        <v>2.4498664614607613</v>
+      </c>
+      <c r="E14">
+        <v>6.0438475571111816</v>
+      </c>
+      <c r="F14">
+        <v>43.615839341589606</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>26</v>
+      </c>
+      <c r="B15">
+        <v>36.078511490621082</v>
+      </c>
+      <c r="D15">
+        <v>1.8595618939661129</v>
+      </c>
+      <c r="E15">
+        <v>5.0848986300286292</v>
+      </c>
+      <c r="F15">
+        <v>43.628240126287153</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="4"/>
+      <c r="C18" s="5"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="7">
+        <v>10</v>
+      </c>
+      <c r="C21">
+        <v>14.325600000000001</v>
+      </c>
+      <c r="G21" s="6">
+        <v>24.688800000000001</v>
+      </c>
+      <c r="H21">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>15</v>
       </c>
-      <c r="C10">
+      <c r="C22">
         <v>20.116800000000001</v>
       </c>
-      <c r="G10">
+      <c r="G22" s="3">
         <v>30.1752</v>
       </c>
+      <c r="H22">
+        <v>16.47</v>
+      </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>16</v>
-      </c>
-      <c r="B11">
-        <v>29.492855410981377</v>
-      </c>
-      <c r="D11">
-        <v>3.6244941391413121</v>
-      </c>
-      <c r="E11">
-        <v>8.5778441065895183</v>
-      </c>
-      <c r="F11">
-        <v>39.486924298506949</v>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>20</v>
+      </c>
+      <c r="C23">
+        <v>20.421600000000002</v>
+      </c>
+      <c r="G23" s="6">
+        <v>31.089600000000001</v>
+      </c>
+      <c r="H23">
+        <v>16.975000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>18</v>
-      </c>
-      <c r="B12">
-        <v>31.876605800476643</v>
-      </c>
-      <c r="D12">
-        <v>3.5814365777583035</v>
-      </c>
-      <c r="E12">
-        <v>8.2172795945172261</v>
-      </c>
-      <c r="F12">
-        <v>41.299882744762179</v>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>25</v>
+      </c>
+      <c r="C24">
+        <v>17.3736</v>
+      </c>
+      <c r="G24" s="3">
+        <v>28.956</v>
+      </c>
+      <c r="H24">
+        <v>16.344000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>20</v>
-      </c>
-      <c r="B13">
-        <v>33.665694816156972</v>
-      </c>
-      <c r="C13">
-        <v>20.421600000000002</v>
-      </c>
-      <c r="D13">
-        <v>3.345700169036423</v>
-      </c>
-      <c r="E13">
-        <v>7.6472604719564963</v>
-      </c>
-      <c r="F13">
-        <v>42.527524768893407</v>
-      </c>
-      <c r="G13">
-        <v>31.089600000000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>22</v>
-      </c>
-      <c r="B14">
-        <v>34.955435729999998</v>
-      </c>
-      <c r="D14">
-        <v>2.9564879576701841</v>
-      </c>
-      <c r="E14">
-        <v>6.9099309450000002</v>
-      </c>
-      <c r="F14">
-        <v>43.271801437912231</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>24</v>
-      </c>
-      <c r="B15">
-        <v>35.820851562722908</v>
-      </c>
-      <c r="D15">
-        <v>2.4498664614607613</v>
-      </c>
-      <c r="E15">
-        <v>6.0438475571111816</v>
-      </c>
-      <c r="F15">
-        <v>43.615839341589606</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>25</v>
-      </c>
-      <c r="C16">
-        <v>17.3736</v>
-      </c>
-      <c r="G16">
-        <v>28.956</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>26</v>
-      </c>
-      <c r="B17">
-        <v>36.078511490621082</v>
-      </c>
-      <c r="D17">
-        <v>1.8595618939661129</v>
-      </c>
-      <c r="E17">
-        <v>5.0848986300286292</v>
-      </c>
-      <c r="F17">
-        <v>43.628240126287153</v>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>30</v>
+      </c>
+      <c r="H25">
+        <v>15.172000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>